<commit_message>
Figure/table revision: age validation, Figures 2-4, Tables 1-2, validation gates
- Figure 5 age validation (scripts 46-47): age x profile support audit,
  age-interaction GAM diagnostics, age-group standardised risks, robustness.
- Revised manuscript figures (48-58): Figure 2 profile RR redesign; Figure 3
  age-specific absolute risks incl. validated hospitalisation age model (H2)
  and standalone panels/legend; Figure 4 count-vs-profile model comparison
  and final within-count risk-difference figure with title/legend docx.
- Tables (59-60): Table 1 with cohort selection/outcome completeness;
  reconciled joint-profile Main Table 2 and individual-condition supplement;
  reconciliation reports (no numerical discrepancies; stale N in old note fixed).
- Validation gates 3.1-3.4 outputs and scripts 11, 23-45 from earlier sessions.
- .gitignore: exclude individual-level data in 01_Data subfolders and large
  per-person/per-draw caches.
</commit_message>
<xml_diff>
--- a/CHIK_MORBID/03_Output/tables/condition_recording_summaries.xlsx
+++ b/CHIK_MORBID/03_Output/tables/condition_recording_summaries.xlsx
@@ -50559,22 +50559,22 @@
         <v>18</v>
       </c>
       <c r="C2" t="n">
-        <v>1075345</v>
+        <v>984304</v>
       </c>
       <c r="D2" t="n">
-        <v>1075177</v>
+        <v>984145</v>
       </c>
       <c r="E2" t="n">
-        <v>0.99984377106882</v>
+        <v>0.999838464539411</v>
       </c>
       <c r="F2" t="n">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="G2" t="n">
-        <v>0.999818295899142</v>
+        <v>0.999811331920989</v>
       </c>
       <c r="H2" t="n">
-        <v>0.999865675063843</v>
+        <v>0.999861695718064</v>
       </c>
     </row>
     <row r="3">
@@ -50611,22 +50611,22 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>1075345</v>
+        <v>984304</v>
       </c>
       <c r="D4" t="n">
-        <v>1075185</v>
+        <v>984154</v>
       </c>
       <c r="E4" t="n">
-        <v>0.999851210541733</v>
+        <v>0.999847608056048</v>
       </c>
       <c r="F4" t="n">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="G4" t="n">
-        <v>0.99982630289176</v>
+        <v>0.999821193961634</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9998725469639</v>
+        <v>0.999870120639324</v>
       </c>
     </row>
     <row r="5">
@@ -50663,22 +50663,22 @@
         <v>18</v>
       </c>
       <c r="C6" t="n">
-        <v>1075345</v>
+        <v>984304</v>
       </c>
       <c r="D6" t="n">
-        <v>1075160</v>
+        <v>984128</v>
       </c>
       <c r="E6" t="n">
-        <v>0.999827962188879</v>
+        <v>0.999821193452429</v>
       </c>
       <c r="F6" t="n">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="G6" t="n">
-        <v>0.999801324062813</v>
+        <v>0.999792756790577</v>
       </c>
       <c r="H6" t="n">
-        <v>0.999851029253239</v>
+        <v>0.999845728809321</v>
       </c>
     </row>
     <row r="7">
@@ -50715,22 +50715,22 @@
         <v>18</v>
       </c>
       <c r="C8" t="n">
-        <v>1075345</v>
+        <v>984304</v>
       </c>
       <c r="D8" t="n">
-        <v>1075154</v>
+        <v>984122</v>
       </c>
       <c r="E8" t="n">
-        <v>0.999822382584194</v>
+        <v>0.999815097774671</v>
       </c>
       <c r="F8" t="n">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="G8" t="n">
-        <v>0.999795346797649</v>
+        <v>0.999786215945627</v>
       </c>
       <c r="H8" t="n">
-        <v>0.999845847348896</v>
+        <v>0.999840078346334</v>
       </c>
     </row>
     <row r="9">
@@ -50767,22 +50767,22 @@
         <v>18</v>
       </c>
       <c r="C10" t="n">
-        <v>1075345</v>
+        <v>984304</v>
       </c>
       <c r="D10" t="n">
-        <v>1075157</v>
+        <v>984125</v>
       </c>
       <c r="E10" t="n">
-        <v>0.999825172386536</v>
+        <v>0.99981814561355</v>
       </c>
       <c r="F10" t="n">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="G10" t="n">
-        <v>0.999798334640563</v>
+        <v>0.999789485439859</v>
       </c>
       <c r="H10" t="n">
-        <v>0.999848439090735</v>
+        <v>0.99984290450607</v>
       </c>
     </row>
     <row r="11">
@@ -50819,22 +50819,22 @@
         <v>18</v>
       </c>
       <c r="C12" t="n">
-        <v>1075345</v>
+        <v>984304</v>
       </c>
       <c r="D12" t="n">
-        <v>1075157</v>
+        <v>984125</v>
       </c>
       <c r="E12" t="n">
-        <v>0.999825172386536</v>
+        <v>0.99981814561355</v>
       </c>
       <c r="F12" t="n">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="G12" t="n">
-        <v>0.999798334640563</v>
+        <v>0.999789485439859</v>
       </c>
       <c r="H12" t="n">
-        <v>0.999848439090735</v>
+        <v>0.99984290450607</v>
       </c>
     </row>
     <row r="13">
@@ -50871,22 +50871,22 @@
         <v>18</v>
       </c>
       <c r="C14" t="n">
-        <v>1075345</v>
+        <v>984304</v>
       </c>
       <c r="D14" t="n">
-        <v>1075148</v>
+        <v>984117</v>
       </c>
       <c r="E14" t="n">
-        <v>0.999816802979509</v>
+        <v>0.999810018043206</v>
       </c>
       <c r="F14" t="n">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="G14" t="n">
-        <v>0.999789375703736</v>
+        <v>0.999780770791427</v>
       </c>
       <c r="H14" t="n">
-        <v>0.999840659273303</v>
+        <v>0.999835364077253</v>
       </c>
     </row>
     <row r="15">

</xml_diff>